<commit_message>
Enhance error handling in Worksheet_extract.py and streamline file path management. Update Inbound_Master.py to ensure compatibility with direct execution by including project root in sys.path.
</commit_message>
<xml_diff>
--- a/J30/Input_files/WorkSheet.xlsx
+++ b/J30/Input_files/WorkSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vgana3/Documents/GitHub/Nike/J30/Input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE32BD62-628C-664B-A9A1-1A2711F0C0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4921F5B2-392F-1F4D-971C-28FFE195A386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateASN" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,20 @@
     <sheet name="SearchASN" sheetId="6" r:id="rId6"/>
     <sheet name="BackUP" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -51,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="63">
   <si>
     <t>Plant</t>
   </si>
@@ -83,9 +96,6 @@
     <t>QA</t>
   </si>
   <si>
-    <t>899371-091-M</t>
-  </si>
-  <si>
     <t>0005005401</t>
   </si>
   <si>
@@ -231,13 +241,25 @@
   </si>
   <si>
     <t>0215056616</t>
+  </si>
+  <si>
+    <t>FQ0462-010-M;FQ0462-010-XL;DV4349-701-3.5Y;DV4351-003-1Y</t>
+  </si>
+  <si>
+    <t>10;20;6;6</t>
+  </si>
+  <si>
+    <t>V01</t>
+  </si>
+  <si>
+    <t>3000;200;240;3900</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -283,6 +305,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -347,9 +375,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -361,6 +386,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -702,7 +728,7 @@
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -744,40 +770,40 @@
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
-        <v>81</v>
+      <c r="C2" t="s">
+        <v>61</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="8">
-        <v>18</v>
-      </c>
-      <c r="G2" s="8">
-        <v>6</v>
-      </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
       <c r="H4" s="3"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="D11" s="12"/>
+      <c r="D11" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -800,33 +826,33 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>19</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="D2" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -844,41 +870,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="13"/>
+        <v>58</v>
+      </c>
+      <c r="D2" s="12"/>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -899,38 +925,38 @@
         <v>1</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
         <v>29</v>
-      </c>
-      <c r="D2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -959,22 +985,22 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>35</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>36</v>
-      </c>
-      <c r="H1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -988,10 +1014,10 @@
         <v>1</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1018,7 +1044,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1029,7 +1055,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1056,19 +1082,19 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
         <v>11</v>
-      </c>
-      <c r="H1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1082,10 +1108,10 @@
         <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
         <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1099,19 +1125,19 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="F3" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
         <v>11</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1125,19 +1151,19 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
         <v>11</v>
-      </c>
-      <c r="H4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1151,44 +1177,44 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="G5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
         <v>11</v>
-      </c>
-      <c r="H5" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="D6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="D7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="D8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="D9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1199,16 +1225,16 @@
         <v>1</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1223,7 +1249,7 @@
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F16" s="4"/>
     </row>
@@ -1239,7 +1265,7 @@
       </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F17" s="4"/>
     </row>
@@ -1255,26 +1281,26 @@
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F18" s="4"/>
     </row>
     <row r="22" spans="1:10">
       <c r="D22" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" t="s">
         <v>55</v>
-      </c>
-      <c r="E22" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="D25" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="D26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:10">

</xml_diff>